<commit_message>
Actualización index.html y Excel
</commit_message>
<xml_diff>
--- a/resources/Comensales.xlsx
+++ b/resources/Comensales.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BOOM\Documents\Programación 1\Corte 2\L26.2.p.c2.18.comensales\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1390F96D-0331-40EE-A04E-3E3810E94CB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33213A3E-47FD-4305-AEBD-4C1531890276}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -185,7 +185,7 @@
     <numFmt numFmtId="164" formatCode="[$$-540A]#,##0"/>
     <numFmt numFmtId="165" formatCode="[$$-409]#,##0"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -224,6 +224,14 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial Unicode MS"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="5">
@@ -318,7 +326,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -390,6 +398,7 @@
     <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -736,6 +745,7 @@
         <v>0</v>
       </c>
       <c r="D1" s="1"/>
+      <c r="E1" s="31"/>
     </row>
     <row r="3" spans="1:14">
       <c r="A3" s="2" t="s">

</xml_diff>